<commit_message>
Update website artifacts with latest graded outputs and dashboards.
Refresh mobile/www and ui_runner web payloads (graded props, slate/ticket eval,
latest json snapshots, and report assets) so the site reflects current grading data.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-04.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-04.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F2" t="n">
         <v>17</v>
       </c>
       <c r="G2" t="n">
-        <v>68.5</v>
+        <v>69.09999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
-        <v>80</v>
+        <v>47.9</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G4" t="n">
-        <v>54.5</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E5" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G5" t="n">
-        <v>70.8</v>
+        <v>71.90000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G6" t="n">
-        <v>52</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="7">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="E8" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F8" t="n">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="G8" t="n">
-        <v>41.7</v>
+        <v>41.3</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="E9" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G9" t="n">
-        <v>60.4</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>568</v>
+        <v>580</v>
       </c>
       <c r="E10" t="n">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F10" t="n">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="G10" t="n">
-        <v>60</v>
+        <v>59.3</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>246</v>
+        <v>322</v>
       </c>
       <c r="E11" t="n">
-        <v>160</v>
+        <v>195</v>
       </c>
       <c r="F11" t="n">
-        <v>86</v>
+        <v>127</v>
       </c>
       <c r="G11" t="n">
-        <v>65</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>225</v>
+        <v>264</v>
       </c>
       <c r="E12" t="n">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="F12" t="n">
-        <v>87</v>
+        <v>115</v>
       </c>
       <c r="G12" t="n">
-        <v>61.3</v>
+        <v>56.4</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>155</v>
+        <v>236</v>
       </c>
       <c r="E13" t="n">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="F13" t="n">
-        <v>71</v>
+        <v>131</v>
       </c>
       <c r="G13" t="n">
-        <v>54.2</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>172</v>
+        <v>232</v>
       </c>
       <c r="E14" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="F14" t="n">
-        <v>127</v>
+        <v>177</v>
       </c>
       <c r="G14" t="n">
-        <v>26.2</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="E15" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F15" t="n">
-        <v>92</v>
+        <v>139</v>
       </c>
       <c r="G15" t="n">
-        <v>21.4</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F16" t="n">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1865</v>
+        <v>3120</v>
       </c>
       <c r="E17" t="n">
-        <v>380</v>
+        <v>511</v>
       </c>
       <c r="F17" t="n">
-        <v>1485</v>
+        <v>2609</v>
       </c>
       <c r="G17" t="n">
-        <v>20.4</v>
+        <v>16.4</v>
       </c>
     </row>
   </sheetData>
@@ -1106,10 +1106,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44</v>
+        <v>40.7</v>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
         <v>40</v>
@@ -1118,37 +1118,40 @@
         <v>35</v>
       </c>
       <c r="F2" t="n">
-        <v>50</v>
+        <v>44.9</v>
       </c>
       <c r="G2" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="H2" t="n">
-        <v>42.5</v>
+        <v>40.5</v>
       </c>
       <c r="I2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J2" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="K2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L2" t="n">
         <v>25</v>
       </c>
-      <c r="K2" t="n">
-        <v>8</v>
-      </c>
-      <c r="L2" t="n">
-        <v>100</v>
-      </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P2" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="Q2" t="n">
-        <v>57</v>
+        <v>120</v>
       </c>
       <c r="R2" t="n">
         <v>54.5</v>
@@ -1159,17 +1162,23 @@
       <c r="U2" t="n">
         <v>0</v>
       </c>
+      <c r="V2" t="n">
+        <v>100</v>
+      </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X2" t="n">
-        <v>24.7</v>
+        <v>24.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>85</v>
+        <v>87</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>42.9</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -1191,10 +1200,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>67.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D3" t="n">
         <v>76.3</v>
@@ -1203,61 +1212,67 @@
         <v>97</v>
       </c>
       <c r="F3" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>89</v>
+      </c>
+      <c r="H3" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>76</v>
+      </c>
+      <c r="J3" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="K3" t="n">
+        <v>52</v>
+      </c>
+      <c r="L3" t="n">
+        <v>30</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N3" t="n">
+        <v>25</v>
+      </c>
+      <c r="O3" t="n">
+        <v>32</v>
+      </c>
+      <c r="P3" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>191</v>
+      </c>
+      <c r="R3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="S3" t="n">
+        <v>26</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
         <v>66.7</v>
       </c>
-      <c r="G3" t="n">
-        <v>78</v>
-      </c>
-      <c r="H3" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>61</v>
-      </c>
-      <c r="J3" t="n">
-        <v>55.3</v>
-      </c>
-      <c r="K3" t="n">
-        <v>38</v>
-      </c>
-      <c r="L3" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="M3" t="n">
-        <v>14</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>54</v>
-      </c>
-      <c r="R3" t="n">
-        <v>68</v>
-      </c>
-      <c r="S3" t="n">
-        <v>25</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0</v>
-      </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X3" t="n">
-        <v>50</v>
+        <v>49.7</v>
       </c>
       <c r="Y3" t="n">
-        <v>180</v>
+        <v>183</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>47.4</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
@@ -1421,29 +1436,50 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
+      <c r="F6" t="n">
+        <v>16.7</v>
+      </c>
       <c r="G6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>28.6</v>
       </c>
       <c r="K6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="N6" t="n">
+        <v>25.7</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>35</v>
+      </c>
+      <c r="P6" t="n">
+        <v>8.1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -1451,14 +1487,23 @@
       <c r="U6" t="n">
         <v>0</v>
       </c>
+      <c r="V6" t="n">
+        <v>50</v>
+      </c>
       <c r="W6" t="n">
+        <v>2</v>
+      </c>
+      <c r="X6" t="n">
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>55.6</v>
       </c>
       <c r="AA6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -1477,88 +1522,88 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60</v>
+        <v>59.3</v>
       </c>
       <c r="C7" t="n">
-        <v>568</v>
+        <v>580</v>
       </c>
       <c r="D7" t="n">
-        <v>65</v>
+        <v>60.6</v>
       </c>
       <c r="E7" t="n">
-        <v>246</v>
+        <v>322</v>
       </c>
       <c r="F7" t="n">
-        <v>61.3</v>
+        <v>56.4</v>
       </c>
       <c r="G7" t="n">
-        <v>225</v>
+        <v>264</v>
       </c>
       <c r="H7" t="n">
-        <v>54.2</v>
+        <v>44.5</v>
       </c>
       <c r="I7" t="n">
-        <v>155</v>
+        <v>236</v>
       </c>
       <c r="J7" t="n">
-        <v>26.2</v>
+        <v>23.7</v>
       </c>
       <c r="K7" t="n">
-        <v>172</v>
+        <v>232</v>
       </c>
       <c r="L7" t="n">
-        <v>21.4</v>
+        <v>17.8</v>
       </c>
       <c r="M7" t="n">
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>20.8</v>
       </c>
       <c r="O7" t="n">
-        <v>8</v>
+        <v>96</v>
       </c>
       <c r="P7" t="n">
-        <v>20.4</v>
+        <v>16.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>1865</v>
+        <v>3120</v>
       </c>
       <c r="R7" t="n">
-        <v>68.5</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="S7" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="T7" t="n">
-        <v>54.5</v>
+        <v>46.4</v>
       </c>
       <c r="U7" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="V7" t="n">
-        <v>52</v>
+        <v>56.2</v>
       </c>
       <c r="W7" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="X7" t="n">
-        <v>41.7</v>
+        <v>41.3</v>
       </c>
       <c r="Y7" t="n">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="Z7" t="n">
-        <v>80</v>
+        <v>47.9</v>
       </c>
       <c r="AA7" t="n">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="AB7" t="n">
-        <v>70.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="AC7" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="AD7" t="n">
         <v>45</v>
@@ -1567,10 +1612,10 @@
         <v>20</v>
       </c>
       <c r="AF7" t="n">
-        <v>60.4</v>
+        <v>62.6</v>
       </c>
       <c r="AG7" t="n">
-        <v>91</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-05-08 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-04.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-04.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E2" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F2" t="n">
         <v>17</v>
       </c>
       <c r="G2" t="n">
-        <v>69.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E3" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F3" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="G3" t="n">
-        <v>47.9</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>46.4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G5" t="n">
-        <v>71.90000000000001</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>14</v>
-      </c>
-      <c r="G6" t="n">
-        <v>56.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="F7" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="G7" t="n">
-        <v>45</v>
+        <v>57.9</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +642,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>380</v>
+        <v>441</v>
       </c>
       <c r="E8" t="n">
-        <v>157</v>
+        <v>189</v>
       </c>
       <c r="F8" t="n">
-        <v>223</v>
+        <v>252</v>
       </c>
       <c r="G8" t="n">
-        <v>41.3</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="E9" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F9" t="n">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="G9" t="n">
-        <v>62.6</v>
+        <v>52.9</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>580</v>
+        <v>596</v>
       </c>
       <c r="E10" t="n">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="F10" t="n">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="G10" t="n">
-        <v>59.3</v>
+        <v>58.7</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>322</v>
+        <v>306</v>
       </c>
       <c r="E11" t="n">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F11" t="n">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="G11" t="n">
-        <v>60.6</v>
+        <v>61.4</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E12" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F12" t="n">
         <v>115</v>
       </c>
       <c r="G12" t="n">
-        <v>56.4</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="13">
@@ -819,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="E14" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F14" t="n">
-        <v>177</v>
+        <v>149</v>
       </c>
       <c r="G14" t="n">
-        <v>23.7</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="E15" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F15" t="n">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="G15" t="n">
-        <v>17.8</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +874,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>96</v>
+        <v>154</v>
       </c>
       <c r="E16" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="F16" t="n">
-        <v>76</v>
+        <v>118</v>
       </c>
       <c r="G16" t="n">
-        <v>20.8</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3120</v>
+        <v>3123</v>
       </c>
       <c r="E17" t="n">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="F17" t="n">
-        <v>2609</v>
+        <v>2614</v>
       </c>
       <c r="G17" t="n">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
     </row>
   </sheetData>
@@ -1142,55 +1139,52 @@
         <v>4</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>7.7</v>
       </c>
       <c r="O2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P2" t="n">
-        <v>12.5</v>
+        <v>12.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="R2" t="n">
-        <v>54.5</v>
+        <v>58.3</v>
       </c>
       <c r="S2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>88</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
         <v>100</v>
       </c>
-      <c r="W2" t="n">
-        <v>2</v>
-      </c>
-      <c r="X2" t="n">
-        <v>24.1</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>87</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>7</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>0</v>
-      </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF2" t="n">
-        <v>37.5</v>
+        <v>35.3</v>
       </c>
       <c r="AG2" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -1224,67 +1218,70 @@
         <v>76</v>
       </c>
       <c r="J3" t="n">
-        <v>42.3</v>
+        <v>41.5</v>
       </c>
       <c r="K3" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="L3" t="n">
-        <v>30</v>
+        <v>27.3</v>
       </c>
       <c r="M3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="N3" t="n">
-        <v>25</v>
+        <v>28.3</v>
       </c>
       <c r="O3" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="P3" t="n">
-        <v>19.4</v>
+        <v>19.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>191</v>
+        <v>208</v>
       </c>
       <c r="R3" t="n">
-        <v>69.2</v>
+        <v>63</v>
       </c>
       <c r="S3" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="T3" t="n">
+        <v>100</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" t="n">
-        <v>66.7</v>
+        <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>49.7</v>
+        <v>50.5</v>
       </c>
       <c r="Y3" t="n">
-        <v>183</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>47.4</v>
+        <v>184</v>
       </c>
       <c r="AA3" t="n">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>40</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>40</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AF3" t="n">
-        <v>38.5</v>
+        <v>48.4</v>
       </c>
       <c r="AG3" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -1373,22 +1370,22 @@
         <v>38</v>
       </c>
       <c r="J5" t="n">
-        <v>29.4</v>
+        <v>35.7</v>
       </c>
       <c r="K5" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="L5" t="n">
-        <v>16.7</v>
+        <v>14.3</v>
       </c>
       <c r="M5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P5" t="n">
         <v>27.8</v>
@@ -1417,17 +1414,23 @@
       <c r="AA5" t="n">
         <v>0</v>
       </c>
+      <c r="AB5" t="n">
+        <v>100</v>
+      </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>71.40000000000001</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AF5" t="n">
-        <v>61.5</v>
+        <v>40</v>
       </c>
       <c r="AG5" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -1440,7 +1443,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -1470,16 +1473,16 @@
         <v>2</v>
       </c>
       <c r="N6" t="n">
-        <v>25.7</v>
+        <v>19.6</v>
       </c>
       <c r="O6" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="P6" t="n">
-        <v>8.1</v>
+        <v>11.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -1487,23 +1490,17 @@
       <c r="U6" t="n">
         <v>0</v>
       </c>
-      <c r="V6" t="n">
-        <v>50</v>
-      </c>
       <c r="W6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="Y6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>55.6</v>
+        <v>3</v>
       </c>
       <c r="AA6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -1511,8 +1508,11 @@
       <c r="AE6" t="n">
         <v>0</v>
       </c>
+      <c r="AF6" t="n">
+        <v>64.3</v>
+      </c>
       <c r="AG6" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1522,22 +1522,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>59.3</v>
+        <v>58.7</v>
       </c>
       <c r="C7" t="n">
-        <v>580</v>
+        <v>596</v>
       </c>
       <c r="D7" t="n">
-        <v>60.6</v>
+        <v>61.4</v>
       </c>
       <c r="E7" t="n">
-        <v>322</v>
+        <v>306</v>
       </c>
       <c r="F7" t="n">
-        <v>56.4</v>
+        <v>56.6</v>
       </c>
       <c r="G7" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H7" t="n">
         <v>44.5</v>
@@ -1546,76 +1546,73 @@
         <v>236</v>
       </c>
       <c r="J7" t="n">
-        <v>23.7</v>
+        <v>24.7</v>
       </c>
       <c r="K7" t="n">
-        <v>232</v>
+        <v>198</v>
       </c>
       <c r="L7" t="n">
-        <v>17.8</v>
+        <v>15.3</v>
       </c>
       <c r="M7" t="n">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="N7" t="n">
-        <v>20.8</v>
+        <v>23.4</v>
       </c>
       <c r="O7" t="n">
-        <v>96</v>
+        <v>154</v>
       </c>
       <c r="P7" t="n">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>3120</v>
+        <v>3123</v>
       </c>
       <c r="R7" t="n">
-        <v>69.09999999999999</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="S7" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T7" t="n">
-        <v>46.4</v>
+        <v>100</v>
       </c>
       <c r="U7" t="n">
-        <v>28</v>
-      </c>
-      <c r="V7" t="n">
-        <v>56.2</v>
+        <v>1</v>
       </c>
       <c r="W7" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>41.3</v>
+        <v>42.9</v>
       </c>
       <c r="Y7" t="n">
-        <v>380</v>
+        <v>441</v>
       </c>
       <c r="Z7" t="n">
-        <v>47.9</v>
+        <v>75</v>
       </c>
       <c r="AA7" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="AB7" t="n">
-        <v>71.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="AC7" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="AD7" t="n">
-        <v>45</v>
+        <v>57.9</v>
       </c>
       <c r="AE7" t="n">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="AF7" t="n">
-        <v>62.6</v>
+        <v>52.9</v>
       </c>
       <c r="AG7" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>